<commit_message>
Datos cuencas ejemplo y carga de Excel
</commit_message>
<xml_diff>
--- a/Data_HU_SCS.xlsx
+++ b/Data_HU_SCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04ED263E-D365-4180-ABF1-FD3EFC6084CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{256F7226-844E-4481-B68C-35B79B550AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{22632642-5EDA-433C-AFAA-A16699809E0D}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22632642-5EDA-433C-AFAA-A16699809E0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Cuenca</t>
   </si>
@@ -93,16 +93,43 @@
   </si>
   <si>
     <t>[m/s]</t>
+  </si>
+  <si>
+    <t>AT_CL_01</t>
+  </si>
+  <si>
+    <t>AT_CL_02</t>
+  </si>
+  <si>
+    <t>AT_CL_03</t>
+  </si>
+  <si>
+    <t>AT_CL_04</t>
+  </si>
+  <si>
+    <t>AT_CL_05</t>
+  </si>
+  <si>
+    <t>AT_CL_06</t>
+  </si>
+  <si>
+    <t>AT_CL_07</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -137,10 +164,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -477,7 +504,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E67CCFD8-5B94-43E5-AFB1-BA27C144B982}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
@@ -485,42 +512,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
+      <c r="A2" s="4"/>
       <c r="B2" s="1" t="s">
         <v>11</v>
       </c>
@@ -550,12 +577,265 @@
       </c>
       <c r="K2" s="1" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>25</v>
+      </c>
+      <c r="C3">
+        <v>78</v>
+      </c>
+      <c r="D3">
+        <v>620</v>
+      </c>
+      <c r="E3">
+        <v>1450</v>
+      </c>
+      <c r="F3">
+        <f>E3-D3</f>
+        <v>830</v>
+      </c>
+      <c r="G3">
+        <v>980</v>
+      </c>
+      <c r="H3">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="I3">
+        <v>11.8</v>
+      </c>
+      <c r="J3">
+        <v>6.4</v>
+      </c>
+      <c r="K3">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>6.8</v>
+      </c>
+      <c r="C4">
+        <v>72</v>
+      </c>
+      <c r="D4">
+        <v>410</v>
+      </c>
+      <c r="E4">
+        <v>1020</v>
+      </c>
+      <c r="F4">
+        <f t="shared" ref="F4:F9" si="0">E4-D4</f>
+        <v>610</v>
+      </c>
+      <c r="G4">
+        <v>690</v>
+      </c>
+      <c r="H4">
+        <v>4.1000000000000002E-2</v>
+      </c>
+      <c r="I4">
+        <v>6.4</v>
+      </c>
+      <c r="J4">
+        <v>3.6</v>
+      </c>
+      <c r="K4">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5">
+        <v>12.5</v>
+      </c>
+      <c r="C5">
+        <v>78</v>
+      </c>
+      <c r="D5">
+        <v>220</v>
+      </c>
+      <c r="E5">
+        <v>880</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="0"/>
+        <v>660</v>
+      </c>
+      <c r="G5">
+        <v>520</v>
+      </c>
+      <c r="H5">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="I5">
+        <v>9.1</v>
+      </c>
+      <c r="J5">
+        <v>5</v>
+      </c>
+      <c r="K5">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="C6">
+        <v>83</v>
+      </c>
+      <c r="D6">
+        <v>95</v>
+      </c>
+      <c r="E6">
+        <v>540</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="0"/>
+        <v>445</v>
+      </c>
+      <c r="G6">
+        <v>280</v>
+      </c>
+      <c r="H6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="I6">
+        <v>12.7</v>
+      </c>
+      <c r="J6">
+        <v>7.2</v>
+      </c>
+      <c r="K6">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7">
+        <v>27.4</v>
+      </c>
+      <c r="C7">
+        <v>70</v>
+      </c>
+      <c r="D7">
+        <v>630</v>
+      </c>
+      <c r="E7">
+        <v>1680</v>
+      </c>
+      <c r="F7">
+        <f>E7-D7</f>
+        <v>1050</v>
+      </c>
+      <c r="G7">
+        <v>1120</v>
+      </c>
+      <c r="H7">
+        <v>3.6999999999999998E-2</v>
+      </c>
+      <c r="I7">
+        <v>14.9</v>
+      </c>
+      <c r="J7">
+        <v>8.1</v>
+      </c>
+      <c r="K7">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8">
+        <v>39.6</v>
+      </c>
+      <c r="C8">
+        <v>76</v>
+      </c>
+      <c r="D8">
+        <v>310</v>
+      </c>
+      <c r="E8">
+        <v>980</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="0"/>
+        <v>670</v>
+      </c>
+      <c r="G8">
+        <v>610</v>
+      </c>
+      <c r="H8">
+        <v>0.02</v>
+      </c>
+      <c r="I8">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="J8">
+        <v>10.4</v>
+      </c>
+      <c r="K8">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9">
+        <v>48.2</v>
+      </c>
+      <c r="C9">
+        <v>88</v>
+      </c>
+      <c r="D9">
+        <v>40</v>
+      </c>
+      <c r="E9">
+        <v>420</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="0"/>
+        <v>380</v>
+      </c>
+      <c r="G9">
+        <v>190</v>
+      </c>
+      <c r="H9">
+        <v>0.01</v>
+      </c>
+      <c r="I9">
+        <v>24.8</v>
+      </c>
+      <c r="J9">
+        <v>13.2</v>
+      </c>
+      <c r="K9">
+        <v>0.8</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:A2"/>
   </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
UPDATE planilla, ahora esta habilitada para macros
</commit_message>
<xml_diff>
--- a/Data_HU_SCS.xlsx
+++ b/Data_HU_SCS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Codigos\HU\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{256F7226-844E-4481-B68C-35B79B550AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB4CE109-2A31-4847-9993-C9CEE4D3A852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22632642-5EDA-433C-AFAA-A16699809E0D}"/>
+    <workbookView minimized="1" xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{22632642-5EDA-433C-AFAA-A16699809E0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
   <si>
     <t>Cuenca</t>
   </si>
@@ -114,6 +114,27 @@
   </si>
   <si>
     <t>AT_CL_07</t>
+  </si>
+  <si>
+    <t>California Culverts Practice</t>
+  </si>
+  <si>
+    <t>Giandotti</t>
+  </si>
+  <si>
+    <t>Normas Españolas</t>
+  </si>
+  <si>
+    <t>Tiempo de Concentración Adoptado</t>
+  </si>
+  <si>
+    <t>[hr]</t>
+  </si>
+  <si>
+    <t>SCS</t>
+  </si>
+  <si>
+    <t>Velocidad Media</t>
   </si>
 </sst>
 </file>
@@ -184,6 +205,73 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/activeX/activeX1.xml><?xml version="1.0" encoding="utf-8"?>
+<ax:ocx xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ax:classid="{D7053240-CE69-11CD-A777-00DD01143C57}" ax:persistence="persistStreamInit" r:id="rId1"/>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>12</xdr:col>
+          <xdr:colOff>53340</xdr:colOff>
+          <xdr:row>0</xdr:row>
+          <xdr:rowOff>15240</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>12</xdr:col>
+          <xdr:colOff>982980</xdr:colOff>
+          <xdr:row>0</xdr:row>
+          <xdr:rowOff>685800</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="1025" name="CommandButton1" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s1025"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000001040000}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr/>
+          </xdr:nvSpPr>
+          <xdr:spPr bwMode="auto">
+            <a:xfrm>
+              <a:off x="0" y="0"/>
+              <a:ext cx="0" cy="0"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:extLst>
+              <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
+                <a14:hiddenLine w="9525">
+                  <a:noFill/>
+                  <a:miter lim="800000"/>
+                  <a:headEnd/>
+                  <a:tailEnd/>
+                </a14:hiddenLine>
+              </a:ext>
+            </a:extLst>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -502,16 +590,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E67CCFD8-5B94-43E5-AFB1-BA27C144B982}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E67CCFD8-5B94-43E5-AFB1-BA27C144B982}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:S9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.77734375" customWidth="1"/>
     <col min="2" max="11" width="12.77734375" customWidth="1"/>
+    <col min="13" max="13" width="14.77734375" customWidth="1"/>
+    <col min="14" max="19" width="12.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="55.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -545,8 +635,26 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="N1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="Q1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="R1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="S1" s="3" t="s">
+        <v>28</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2" s="4"/>
       <c r="B2" s="1" t="s">
         <v>11</v>
@@ -578,8 +686,26 @@
       <c r="K2" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="N2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="S2" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>18</v>
       </c>
@@ -615,7 +741,7 @@
         <v>1.2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -651,7 +777,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -687,7 +813,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -723,7 +849,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -759,7 +885,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>23</v>
       </c>
@@ -795,7 +921,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>24</v>
       </c>
@@ -837,5 +963,34 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
+  <controls>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <control shapeId="1025" r:id="rId3" name="CommandButton1">
+          <controlPr defaultSize="0" autoLine="0" r:id="rId4">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>12</xdr:col>
+                <xdr:colOff>53340</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>15240</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>12</xdr:col>
+                <xdr:colOff>982980</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>685800</xdr:rowOff>
+              </to>
+            </anchor>
+          </controlPr>
+        </control>
+      </mc:Choice>
+      <mc:Fallback>
+        <control shapeId="1025" r:id="rId3" name="CommandButton1"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </controls>
 </worksheet>
 </file>
</xml_diff>